<commit_message>
added multilingual support (italian, spanish, french, german, on top of the existing english)
</commit_message>
<xml_diff>
--- a/finance-tracker-SAMPLE.xlsx
+++ b/finance-tracker-SAMPLE.xlsx
@@ -539,7 +539,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D35"/>
+  <dimension ref="A1:D36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -599,377 +599,390 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Owner</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Sample User</t>
-        </is>
-      </c>
+          <t>Language</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr"/>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>shown in the header; blank to hide</t>
+          <t>UI language: en, it, es, fr or de. Blank = follow the browser</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Sample User</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>shown in the header; blank to hide</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
           <t>History from</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
-      <c r="D7" s="2" t="inlineStr">
+      <c r="B8" t="inlineStr"/>
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>YYYY-MM — trims the long-run charts; blank = all data</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="1" t="inlineStr">
-        <is>
-          <t>WEALTH GROUPS</t>
-        </is>
-      </c>
-      <c r="D9" s="2" t="inlineStr">
-        <is>
-          <t>groups INVESTMENTS lines into the wealth donut</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="inlineStr">
         <is>
+          <t>WEALTH GROUPS</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>groups INVESTMENTS lines into the wealth donut</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
           <t>Match (investment name contains; comma-separated)</t>
         </is>
       </c>
-      <c r="B10" s="1" t="inlineStr">
+      <c r="B11" s="1" t="inlineStr">
         <is>
           <t>Label</t>
         </is>
       </c>
-      <c r="C10" s="1" t="inlineStr">
+      <c r="C11" s="1" t="inlineStr">
         <is>
           <t>Colour</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>home,property</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>#5b9cf6</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>pension,sipp</t>
+          <t>home,property</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Pension</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>#f59e0b</t>
+          <t>#5b9cf6</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>pension,sipp</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Pension</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>#f59e0b</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>company,stake,equity</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="B14" t="inlineStr">
         <is>
           <t>Company / business</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr">
+      <c r="C14" t="inlineStr">
         <is>
           <t>#a78bfa</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="1" t="inlineStr">
-        <is>
-          <t>CATEGORIES</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>pins colour and display order; omitted categories still appear</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="inlineStr">
         <is>
+          <t>CATEGORIES</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>pins colour and display order; omitted categories still appear</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B16" s="1" t="inlineStr">
+      <c r="B17" s="1" t="inlineStr">
         <is>
           <t>Colour</t>
         </is>
       </c>
-      <c r="C16" s="1" t="inlineStr">
+      <c r="C17" s="1" t="inlineStr">
         <is>
           <t>Order</t>
         </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>Home</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>#5b9cf6</t>
-        </is>
-      </c>
-      <c r="C17" t="n">
-        <v>1</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Transport</t>
+          <t>Home</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>#2dd4bf</t>
+          <t>#5b9cf6</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Me</t>
+          <t>Transport</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>#4ade80</t>
+          <t>#2dd4bf</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Fun</t>
+          <t>Me</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>#a78bfa</t>
+          <t>#4ade80</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Food drinks out</t>
+          <t>Fun</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>#f472b6</t>
+          <t>#a78bfa</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Family</t>
+          <t>Food drinks out</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>#f87171</t>
+          <t>#f472b6</t>
         </is>
       </c>
       <c r="C22" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>Family</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>#f87171</t>
+        </is>
+      </c>
+      <c r="C23" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
           <t>Work</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="B24" t="inlineStr">
         <is>
           <t>#fbbf24</t>
         </is>
       </c>
-      <c r="C23" t="n">
+      <c r="C24" t="n">
         <v>7</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="1" t="inlineStr">
-        <is>
-          <t>ACCOUNT GROUPS</t>
-        </is>
-      </c>
-      <c r="D25" s="2" t="inlineStr">
-        <is>
-          <t>role 'card repayment' = a bill that clears a card, not a purchase</t>
-        </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="1" t="inlineStr">
         <is>
+          <t>ACCOUNT GROUPS</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="inlineStr">
+        <is>
+          <t>role 'card repayment' = a bill that clears a card, not a purchase</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="1" t="inlineStr">
+        <is>
           <t>Match (bill name contains; comma-separated)</t>
         </is>
       </c>
-      <c r="B26" s="1" t="inlineStr">
+      <c r="B27" s="1" t="inlineStr">
         <is>
           <t>Role</t>
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
+    <row r="28">
+      <c r="A28" t="inlineStr">
         <is>
           <t>card,credit</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr">
+      <c r="B28" t="inlineStr">
         <is>
           <t>card repayment</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" s="1" t="inlineStr">
-        <is>
-          <t>THRESHOLDS</t>
-        </is>
-      </c>
-      <c r="D29" s="2" t="inlineStr">
-        <is>
-          <t>tune when the dashboard warns you</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="inlineStr">
         <is>
+          <t>THRESHOLDS</t>
+        </is>
+      </c>
+      <c r="D30" s="2" t="inlineStr">
+        <is>
+          <t>tune when the dashboard warns you</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="1" t="inlineStr">
+        <is>
           <t>Name</t>
         </is>
       </c>
-      <c r="B30" s="1" t="inlineStr">
+      <c r="B31" s="1" t="inlineStr">
         <is>
           <t>Value</t>
-        </is>
-      </c>
-    </row>
-    <row r="31">
-      <c r="A31" t="inlineStr">
-        <is>
-          <t>Runway warning months</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>2</v>
-      </c>
-      <c r="D31" s="2" t="inlineStr">
-        <is>
-          <t>fewer months of liquid runway than this -&gt; amber</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>Pace warning pct</t>
+          <t>Runway warning months</t>
         </is>
       </c>
       <c r="B32" t="n">
-        <v>100</v>
+        <v>2</v>
       </c>
       <c r="D32" s="2" t="inlineStr">
         <is>
-          <t>spend vs day-proportional budget -&gt; amber</t>
+          <t>fewer months of liquid runway than this -&gt; amber</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Pace alert pct</t>
+          <t>Pace warning pct</t>
         </is>
       </c>
       <c r="B33" t="n">
-        <v>110</v>
+        <v>100</v>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>-&gt; red</t>
+          <t>spend vs day-proportional budget -&gt; amber</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Insight min spend</t>
+          <t>Pace alert pct</t>
         </is>
       </c>
       <c r="B34" t="n">
-        <v>40</v>
+        <v>110</v>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>ignore categories smaller than this when detecting changes</t>
+          <t>-&gt; red</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>Insight min spend</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>40</v>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>ignore categories smaller than this when detecting changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
           <t>Insight min change pct</t>
         </is>
       </c>
-      <c r="B35" t="n">
+      <c r="B36" t="n">
         <v>15</v>
       </c>
-      <c r="D35" s="2" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>only report a change bigger than this</t>
         </is>
@@ -1006,7 +1019,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
     </row>
     <row r="4">
@@ -1328,7 +1341,7 @@
         <v>3200</v>
       </c>
       <c r="E28" s="3" t="n">
-        <v>46257</v>
+        <v>46258</v>
       </c>
     </row>
     <row r="29">
@@ -1349,7 +1362,7 @@
         <v>2400</v>
       </c>
       <c r="E29" s="3" t="n">
-        <v>46272</v>
+        <v>46273</v>
       </c>
     </row>
     <row r="30">
@@ -1370,7 +1383,7 @@
         <v>5000</v>
       </c>
       <c r="E30" s="3" t="n">
-        <v>46432</v>
+        <v>46433</v>
       </c>
     </row>
     <row r="31">
@@ -1391,7 +1404,7 @@
         <v>260000</v>
       </c>
       <c r="E31" s="3" t="n">
-        <v>52802</v>
+        <v>52803</v>
       </c>
     </row>
     <row r="33">
@@ -1556,7 +1569,7 @@
         <v>46234</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1583,7 +1596,7 @@
         <v>46234</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1610,7 +1623,7 @@
         <v>46234</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
@@ -1637,7 +1650,7 @@
         <v>46234</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
@@ -1664,7 +1677,7 @@
         <v>46237</v>
       </c>
       <c r="F8" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -1691,7 +1704,7 @@
         <v>46237</v>
       </c>
       <c r="F9" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
@@ -1718,7 +1731,7 @@
         <v>46242</v>
       </c>
       <c r="F10" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H10" t="inlineStr"/>
     </row>
@@ -1741,7 +1754,7 @@
         <v>46250</v>
       </c>
       <c r="F11" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
@@ -1768,7 +1781,7 @@
         <v>46258</v>
       </c>
       <c r="F12" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
@@ -1795,7 +1808,7 @@
         <v>46262</v>
       </c>
       <c r="F13" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H13" t="inlineStr"/>
     </row>
@@ -1818,7 +1831,7 @@
         <v>46262</v>
       </c>
       <c r="F14" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
@@ -1845,7 +1858,7 @@
         <v>46253</v>
       </c>
       <c r="F15" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H15" t="inlineStr"/>
     </row>
@@ -3236,7 +3249,7 @@
     </row>
     <row r="11">
       <c r="A11" s="3" t="n">
-        <v>46232</v>
+        <v>46233</v>
       </c>
       <c r="B11" t="n">
         <v>18085</v>

</xml_diff>